<commit_message>
adiciona leitura de arquivos e gravacao tabela
</commit_message>
<xml_diff>
--- a/ID01_2_ConcEst_TratarDados/resources/config/Config.xlsx
+++ b/ID01_2_ConcEst_TratarDados/resources/config/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\RPA\ID01_2_ConcEst_TratarDados\ID01_2_ConcEst_TratarDados\resources\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42B8488F-9686-490F-BEA7-8522A3A69EFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90007CA9-0AD8-4F87-986F-D1C87CD87B9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="119">
   <si>
     <t>Name</t>
   </si>
@@ -441,6 +441,15 @@
       </rPr>
       <t>xlsx</t>
     </r>
+  </si>
+  <si>
+    <t>ARQUIVOS BAIXADOS</t>
+  </si>
+  <si>
+    <t>arquivos_baixados</t>
+  </si>
+  <si>
+    <t>C:\Armazenamento\ID01_1_ConcEst_Download\Arquivos_Baixados</t>
   </si>
 </sst>
 </file>
@@ -1466,10 +1475,19 @@
       </c>
     </row>
     <row r="54" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="7"/>
+      <c r="A54" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="B54" s="11"/>
+      <c r="C54" s="12"/>
     </row>
     <row r="55" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55"/>
+      <c r="A55" t="s">
+        <v>117</v>
+      </c>
+      <c r="B55" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="56" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56"/>

</xml_diff>

<commit_message>
adiciona tratamento dados estruturados
</commit_message>
<xml_diff>
--- a/ID01_2_ConcEst_TratarDados/resources/config/Config.xlsx
+++ b/ID01_2_ConcEst_TratarDados/resources/config/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\RPA\ID01_2_ConcEst_TratarDados\ID01_2_ConcEst_TratarDados\resources\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90007CA9-0AD8-4F87-986F-D1C87CD87B9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0DE4C9E-DCE6-4FE1-B460-58E44EDD2E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="122">
   <si>
     <t>Name</t>
   </si>
@@ -450,6 +450,15 @@
   </si>
   <si>
     <t>C:\Armazenamento\ID01_1_ConcEst_Download\Arquivos_Baixados</t>
+  </si>
+  <si>
+    <t>CaminhoBancoLanctoRPS</t>
+  </si>
+  <si>
+    <t>C:\Armazenamento\ID01_3_ConcEst_LanctoRPS\Banco Dados\banco_dados.db</t>
+  </si>
+  <si>
+    <t>Caminho Banco LançtoRPS</t>
   </si>
 </sst>
 </file>
@@ -894,7 +903,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:Z990"/>
+  <dimension ref="A1:Z991"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43.5703125" bestFit="1" customWidth="1"/>
@@ -1105,395 +1114,403 @@
     </row>
     <row r="14" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>32</v>
+        <v>119</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>17</v>
+        <v>120</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>33</v>
+        <v>121</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="7"/>
-      <c r="C15" s="5" t="s">
+      <c r="B16" s="7"/>
+      <c r="C16" s="5" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+    <row r="17" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="12"/>
-    </row>
-    <row r="17" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="B17" s="11"/>
+      <c r="C17" s="12"/>
+    </row>
+    <row r="18" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>37</v>
-      </c>
-      <c r="B17" s="7"/>
-      <c r="C17" s="5" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>38</v>
       </c>
       <c r="B18" s="7"/>
       <c r="C18" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" s="7"/>
+      <c r="C19" s="5" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
+    <row r="20" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="11"/>
-      <c r="C19" s="12"/>
-    </row>
-    <row r="20" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>41</v>
-      </c>
+      <c r="B20" s="11"/>
+      <c r="C20" s="12"/>
     </row>
     <row r="21" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B22" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C22" s="5" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
+    <row r="23" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="B22" s="11"/>
-      <c r="C22" s="12"/>
-    </row>
-    <row r="23" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>46</v>
-      </c>
+      <c r="B23" s="11"/>
+      <c r="C23" s="12"/>
     </row>
     <row r="24" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B25" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="C24" s="2"/>
-    </row>
-    <row r="25" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="10" t="s">
+      <c r="C25" s="2"/>
+    </row>
+    <row r="26" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B25" s="11"/>
-      <c r="C25" s="12"/>
-    </row>
-    <row r="26" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B26" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>49</v>
-      </c>
+      <c r="B26" s="11"/>
+      <c r="C26" s="12"/>
     </row>
     <row r="27" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B27" s="8"/>
+        <v>48</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>17</v>
+      </c>
       <c r="C27" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>53</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="B28" s="8"/>
       <c r="C28" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B29" s="7">
+      <c r="B30" s="7">
         <v>587</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C30" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="10" t="s">
+    <row r="31" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="B30" s="11"/>
-      <c r="C30" s="12"/>
-    </row>
-    <row r="31" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>58</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C31" t="s">
-        <v>59</v>
-      </c>
+      <c r="B31" s="11"/>
+      <c r="C31" s="12"/>
     </row>
     <row r="32" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B32" s="7" t="s">
-        <v>111</v>
+        <v>58</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>17</v>
       </c>
       <c r="C32" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>17</v>
+        <v>111</v>
       </c>
       <c r="C33" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>64</v>
-      </c>
-      <c r="B34" s="7"/>
+        <v>62</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>17</v>
+      </c>
       <c r="C34" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>66</v>
-      </c>
-      <c r="B35" s="7" t="s">
-        <v>17</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="B35" s="7"/>
       <c r="C35" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>66</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C36" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>68</v>
       </c>
-      <c r="B36" s="7"/>
-      <c r="C36" t="s">
+      <c r="B37" s="7"/>
+      <c r="C37" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="10" t="s">
+    <row r="38" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="B37" s="11"/>
-      <c r="C37" s="12"/>
-    </row>
-    <row r="38" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+      <c r="B38" s="11"/>
+      <c r="C38" s="12"/>
+    </row>
+    <row r="39" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>71</v>
       </c>
-      <c r="B38" s="7" t="s">
+      <c r="B39" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C39" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="10" t="s">
+    <row r="40" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B39" s="11"/>
-      <c r="C39" s="12"/>
-    </row>
-    <row r="40" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+      <c r="B40" s="11"/>
+      <c r="C40" s="12"/>
+    </row>
+    <row r="41" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>74</v>
       </c>
-      <c r="B40" s="7" t="s">
+      <c r="B41" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C41" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="10" t="s">
+    <row r="42" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B41" s="11"/>
-      <c r="C41" s="12"/>
-    </row>
-    <row r="42" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>77</v>
-      </c>
-      <c r="B42" s="4"/>
-      <c r="C42" s="2" t="s">
-        <v>78</v>
-      </c>
+      <c r="B42" s="11"/>
+      <c r="C42" s="12"/>
     </row>
     <row r="43" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>79</v>
+      </c>
+      <c r="B44" s="4"/>
+      <c r="C44" s="2" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="10" t="s">
+    <row r="45" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="B44" s="11"/>
-      <c r="C44" s="12"/>
-    </row>
-    <row r="45" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B45" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>83</v>
-      </c>
+      <c r="B45" s="11"/>
+      <c r="C45" s="12"/>
     </row>
     <row r="46" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B46" s="7"/>
+        <v>82</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>17</v>
+      </c>
       <c r="C46" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B47" s="7" t="s">
-        <v>17</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="B47" s="7"/>
       <c r="C47" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B48" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B48" s="7"/>
-      <c r="C48" s="2" t="s">
+      <c r="B49" s="7"/>
+      <c r="C49" s="2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="10" t="s">
+    <row r="50" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B49" s="11"/>
-      <c r="C49" s="12"/>
-    </row>
-    <row r="50" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>90</v>
-      </c>
-      <c r="B50" t="s">
-        <v>101</v>
-      </c>
-      <c r="C50" t="s">
-        <v>91</v>
-      </c>
+      <c r="B50" s="11"/>
+      <c r="C50" s="12"/>
     </row>
     <row r="51" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>90</v>
+      </c>
+      <c r="B51" t="s">
+        <v>101</v>
+      </c>
+      <c r="C51" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>92</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B52" t="s">
         <v>102</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C52" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="10" t="s">
+    <row r="53" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="B52" s="11"/>
-      <c r="C52" s="12"/>
-    </row>
-    <row r="53" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
+      <c r="B53" s="11"/>
+      <c r="C53" s="12"/>
+    </row>
+    <row r="54" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
         <v>114</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B54" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="10" t="s">
+    <row r="55" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="B54" s="11"/>
-      <c r="C54" s="12"/>
-    </row>
-    <row r="55" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+      <c r="B55" s="11"/>
+      <c r="C55" s="12"/>
+    </row>
+    <row r="56" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
         <v>117</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B56" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56"/>
-    </row>
     <row r="57" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="7"/>
+      <c r="B57"/>
     </row>
     <row r="58" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="7"/>
@@ -1510,8 +1527,8 @@
     <row r="62" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="7"/>
     </row>
-    <row r="63" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="4"/>
+    <row r="63" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B63" s="7"/>
     </row>
     <row r="64" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B64" s="4"/>
@@ -4293,6 +4310,9 @@
     </row>
     <row r="990" spans="2:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B990" s="4"/>
+    </row>
+    <row r="991" spans="2:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B991" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
adiciona logica de criacao da fila Performer
</commit_message>
<xml_diff>
--- a/ID01_2_ConcEst_TratarDados/resources/config/Config.xlsx
+++ b/ID01_2_ConcEst_TratarDados/resources/config/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\RPA\ID01_2_ConcEst_TratarDados\ID01_2_ConcEst_TratarDados\resources\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0DE4C9E-DCE6-4FE1-B460-58E44EDD2E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37C90D03-0ABD-4F3D-9EFD-640F44AF74A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="123">
   <si>
     <t>Name</t>
   </si>
@@ -459,6 +459,9 @@
   </si>
   <si>
     <t>Caminho Banco LançtoRPS</t>
+  </si>
+  <si>
+    <t>tbl_Fila_Proc_Performer</t>
   </si>
 </sst>
 </file>
@@ -1163,7 +1166,9 @@
       <c r="A19" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B19" s="7"/>
+      <c r="B19" t="s">
+        <v>122</v>
+      </c>
       <c r="C19" s="5" t="s">
         <v>97</v>
       </c>

</xml_diff>